<commit_message>
feat: add projectile restraint damage
</commit_message>
<xml_diff>
--- a/config/excel/Unit.xlsx
+++ b/config/excel/Unit.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MyZiegler\github\ra2\config\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12E5BE0B-9C43-43B6-BA61-293B969F1BF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5503F969-4118-4E15-BE3F-29B40DA0F825}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5070" yWindow="5070" windowWidth="30885" windowHeight="16065" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="960" yWindow="1575" windowWidth="30885" windowHeight="16065" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ConfUnit" sheetId="1" r:id="rId1"/>
     <sheet name="ConfProjectile" sheetId="2" r:id="rId2"/>
+    <sheet name="ConfRestraint" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="93">
   <si>
     <t>ID</t>
   </si>
@@ -376,13 +377,49 @@
   <si>
     <t>（獾式坦克）机枪子弹</t>
     <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Name</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>类型</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>大兵</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>獾式坦克</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>灰熊坦克</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>Infantry</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>BadgerTank</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>GrizzlyTank</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>string</t>
+    <phoneticPr fontId="7" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -434,8 +471,22 @@
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -451,6 +502,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -495,7 +552,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -543,6 +600,21 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1025,7 +1097,7 @@
         <v>63</v>
       </c>
       <c r="E4" s="4">
-        <v>300</v>
+        <v>120</v>
       </c>
       <c r="F4" s="4">
         <v>100</v>
@@ -1034,7 +1106,7 @@
         <v>1</v>
       </c>
       <c r="H4" s="15">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="I4" s="4">
         <v>10</v>
@@ -1043,7 +1115,7 @@
         <v>1</v>
       </c>
       <c r="K4" s="4">
-        <v>5000</v>
+        <v>10000</v>
       </c>
       <c r="L4" s="4">
         <v>1</v>
@@ -1084,7 +1156,7 @@
         <v>64</v>
       </c>
       <c r="E5" s="4">
-        <v>2000</v>
+        <v>250</v>
       </c>
       <c r="F5" s="4">
         <v>100</v>
@@ -1093,7 +1165,7 @@
         <v>3</v>
       </c>
       <c r="H5" s="15">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="I5" s="4">
         <v>10</v>
@@ -1102,7 +1174,7 @@
         <v>2</v>
       </c>
       <c r="K5" s="4">
-        <v>5000</v>
+        <v>12000</v>
       </c>
       <c r="L5" s="4">
         <v>1</v>
@@ -1120,7 +1192,7 @@
         <v>300</v>
       </c>
       <c r="Q5" s="4">
-        <v>80</v>
+        <v>50</v>
       </c>
       <c r="R5" s="4" t="s">
         <v>22</v>
@@ -1143,7 +1215,7 @@
         <v>65</v>
       </c>
       <c r="E6" s="4">
-        <v>3000</v>
+        <v>600</v>
       </c>
       <c r="F6" s="4">
         <v>100</v>
@@ -1152,7 +1224,7 @@
         <v>7</v>
       </c>
       <c r="H6" s="15">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="I6" s="4">
         <v>15</v>
@@ -1161,7 +1233,7 @@
         <v>3</v>
       </c>
       <c r="K6" s="4">
-        <v>20000</v>
+        <v>15000</v>
       </c>
       <c r="L6" s="4">
         <v>1</v>
@@ -1179,7 +1251,7 @@
         <v>500</v>
       </c>
       <c r="Q6" s="4">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="R6" s="4" t="s">
         <v>21</v>
@@ -1351,7 +1423,7 @@
         <v>0</v>
       </c>
       <c r="I4" s="2">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="J4" s="2" t="s">
         <v>42</v>
@@ -1389,7 +1461,7 @@
         <v>0</v>
       </c>
       <c r="I5" s="2">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="J5" s="2" t="s">
         <v>43</v>
@@ -1427,7 +1499,7 @@
         <v>0</v>
       </c>
       <c r="I6" s="2">
-        <v>200</v>
+        <v>80</v>
       </c>
       <c r="J6" s="2" t="s">
         <v>41</v>
@@ -1481,4 +1553,122 @@
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5815676E-82BE-4DAD-8351-2F2C0D1B67AF}">
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
+  <cols>
+    <col min="3" max="3" width="12.625" customWidth="1"/>
+    <col min="4" max="4" width="13.375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="15" x14ac:dyDescent="0.15">
+      <c r="A1" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="18" t="s">
+        <v>84</v>
+      </c>
+      <c r="C1" s="18" t="s">
+        <v>89</v>
+      </c>
+      <c r="D1" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="E1" s="18" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="15" x14ac:dyDescent="0.15">
+      <c r="A2" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" s="18" t="s">
+        <v>92</v>
+      </c>
+      <c r="C2" s="18" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" s="18" t="s">
+        <v>37</v>
+      </c>
+      <c r="E2" s="18" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="15" x14ac:dyDescent="0.15">
+      <c r="A3" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="18" t="s">
+        <v>85</v>
+      </c>
+      <c r="C3" s="20" t="s">
+        <v>86</v>
+      </c>
+      <c r="D3" s="20" t="s">
+        <v>87</v>
+      </c>
+      <c r="E3" s="20" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A4" s="16">
+        <v>1</v>
+      </c>
+      <c r="B4" s="17" t="s">
+        <v>86</v>
+      </c>
+      <c r="C4" s="16">
+        <v>10000</v>
+      </c>
+      <c r="D4" s="16">
+        <v>4000</v>
+      </c>
+      <c r="E4" s="16">
+        <v>16000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A5" s="16">
+        <v>2</v>
+      </c>
+      <c r="B5" s="17" t="s">
+        <v>87</v>
+      </c>
+      <c r="C5" s="16">
+        <v>20000</v>
+      </c>
+      <c r="D5" s="16">
+        <v>10000</v>
+      </c>
+      <c r="E5" s="16">
+        <v>7000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A6" s="16">
+        <v>3</v>
+      </c>
+      <c r="B6" s="17" t="s">
+        <v>88</v>
+      </c>
+      <c r="C6" s="16">
+        <v>9000</v>
+      </c>
+      <c r="D6" s="16">
+        <v>15000</v>
+      </c>
+      <c r="E6" s="16">
+        <v>10000</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="6" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Update unit ranges and pinch zoom handling
</commit_message>
<xml_diff>
--- a/config/excel/Unit.xlsx
+++ b/config/excel/Unit.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MyZiegler\github\ra2\config\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5503F969-4118-4E15-BE3F-29B40DA0F825}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D74C72C3-E6D0-4746-8E2E-D532B82DEB8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="960" yWindow="1575" windowWidth="30885" windowHeight="16065" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="95">
   <si>
     <t>ID</t>
   </si>
@@ -413,6 +413,14 @@
   <si>
     <t>string</t>
     <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>WarningRange</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>预警范围</t>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -552,7 +560,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -614,6 +622,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -883,7 +897,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:S6"/>
+  <dimension ref="A1:T6"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="2" max="2" width="13.125" customWidth="1"/>
@@ -893,20 +907,21 @@
     <col min="6" max="6" width="10.625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="6.25" customWidth="1"/>
     <col min="8" max="8" width="5.5" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15.75" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.5" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.25" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.25" customWidth="1"/>
-    <col min="14" max="14" width="12.375" customWidth="1"/>
-    <col min="15" max="15" width="15.125" customWidth="1"/>
-    <col min="16" max="16" width="12.75" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="14.625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9.25" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="44.625" customWidth="1"/>
+    <col min="9" max="9" width="15.25" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.75" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.5" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.25" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.25" customWidth="1"/>
+    <col min="15" max="15" width="12.375" customWidth="1"/>
+    <col min="16" max="16" width="15.125" customWidth="1"/>
+    <col min="17" max="17" width="12.75" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="14.625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.25" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="44.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:20" ht="15" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -931,41 +946,44 @@
       <c r="H1" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="21" t="s">
+        <v>93</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="L1" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="M1" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="P1" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="P1" s="3" t="s">
+      <c r="Q1" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="R1" s="3" t="s">
+      <c r="S1" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="S1" s="3" t="s">
+      <c r="T1" s="3" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:19" ht="15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:20" ht="15" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>8</v>
       </c>
@@ -990,41 +1008,44 @@
       <c r="H2" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="I2" s="21" t="s">
         <v>8</v>
       </c>
       <c r="J2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="K2" s="3" t="s">
+      <c r="K2" s="1" t="s">
         <v>8</v>
       </c>
       <c r="L2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="M2" s="1" t="s">
+      <c r="M2" s="3" t="s">
         <v>8</v>
       </c>
       <c r="N2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="O2" s="3" t="s">
+      <c r="O2" s="1" t="s">
         <v>8</v>
       </c>
       <c r="P2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="Q2" s="1" t="s">
+      <c r="Q2" s="3" t="s">
         <v>8</v>
       </c>
       <c r="R2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="S2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="S2" s="1" t="s">
+      <c r="T2" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:19" ht="60" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:20" ht="60" x14ac:dyDescent="0.15">
       <c r="A3" s="5" t="s">
         <v>4</v>
       </c>
@@ -1049,41 +1070,44 @@
       <c r="H3" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="I3" s="6" t="s">
+      <c r="I3" s="22" t="s">
+        <v>94</v>
+      </c>
+      <c r="J3" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="J3" s="6" t="s">
+      <c r="K3" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="K3" s="6" t="s">
+      <c r="L3" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="L3" s="11" t="s">
+      <c r="M3" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="M3" s="6" t="s">
+      <c r="N3" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="N3" s="6" t="s">
+      <c r="O3" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="O3" s="6" t="s">
+      <c r="P3" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="P3" s="11" t="s">
+      <c r="Q3" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="Q3" s="6" t="s">
+      <c r="R3" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="R3" s="7" t="s">
+      <c r="S3" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="S3" s="7" t="s">
+      <c r="T3" s="7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:19" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:20" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
         <v>1</v>
       </c>
@@ -1108,41 +1132,44 @@
       <c r="H4" s="15">
         <v>0</v>
       </c>
-      <c r="I4" s="4">
-        <v>10</v>
+      <c r="I4" s="15">
+        <v>20</v>
       </c>
       <c r="J4" s="4">
+        <v>12</v>
+      </c>
+      <c r="K4" s="4">
         <v>1</v>
       </c>
-      <c r="K4" s="4">
+      <c r="L4" s="4">
         <v>10000</v>
       </c>
-      <c r="L4" s="4">
+      <c r="M4" s="4">
         <v>1</v>
-      </c>
-      <c r="M4" s="4">
-        <v>10000</v>
       </c>
       <c r="N4" s="4">
         <v>10000</v>
       </c>
       <c r="O4" s="4">
+        <v>10000</v>
+      </c>
+      <c r="P4" s="4">
         <v>30000</v>
       </c>
-      <c r="P4" s="4">
+      <c r="Q4" s="4">
         <v>100</v>
       </c>
-      <c r="Q4" s="4">
+      <c r="R4" s="4">
         <v>20</v>
       </c>
-      <c r="R4" s="4" t="s">
+      <c r="S4" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="S4" s="4" t="s">
+      <c r="T4" s="4" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="1:19" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:20" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
         <v>2</v>
       </c>
@@ -1167,41 +1194,44 @@
       <c r="H5" s="15">
         <v>0</v>
       </c>
-      <c r="I5" s="4">
-        <v>10</v>
+      <c r="I5" s="15">
+        <v>20</v>
       </c>
       <c r="J5" s="4">
+        <v>20</v>
+      </c>
+      <c r="K5" s="4">
         <v>2</v>
       </c>
-      <c r="K5" s="4">
+      <c r="L5" s="4">
         <v>12000</v>
       </c>
-      <c r="L5" s="4">
+      <c r="M5" s="4">
         <v>1</v>
       </c>
-      <c r="M5" s="4">
+      <c r="N5" s="4">
         <v>8000</v>
       </c>
-      <c r="N5" s="4">
+      <c r="O5" s="4">
         <v>15000</v>
       </c>
-      <c r="O5" s="4">
+      <c r="P5" s="4">
         <v>60000</v>
       </c>
-      <c r="P5" s="4">
+      <c r="Q5" s="4">
         <v>300</v>
       </c>
-      <c r="Q5" s="4">
+      <c r="R5" s="4">
         <v>50</v>
       </c>
-      <c r="R5" s="4" t="s">
+      <c r="S5" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="S5" s="4" t="s">
+      <c r="T5" s="4" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="6" spans="1:19" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:20" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
         <v>3</v>
       </c>
@@ -1226,37 +1256,40 @@
       <c r="H6" s="15">
         <v>0</v>
       </c>
-      <c r="I6" s="4">
-        <v>15</v>
+      <c r="I6" s="15">
+        <v>20</v>
       </c>
       <c r="J6" s="4">
+        <v>24</v>
+      </c>
+      <c r="K6" s="4">
         <v>3</v>
       </c>
-      <c r="K6" s="4">
+      <c r="L6" s="4">
         <v>15000</v>
       </c>
-      <c r="L6" s="4">
+      <c r="M6" s="4">
         <v>1</v>
       </c>
-      <c r="M6" s="4">
+      <c r="N6" s="4">
         <v>10000</v>
       </c>
-      <c r="N6" s="4">
+      <c r="O6" s="4">
         <v>20000</v>
       </c>
-      <c r="O6" s="4">
+      <c r="P6" s="4">
         <v>50000</v>
       </c>
-      <c r="P6" s="4">
+      <c r="Q6" s="4">
         <v>500</v>
       </c>
-      <c r="Q6" s="4">
+      <c r="R6" s="4">
         <v>80</v>
       </c>
-      <c r="R6" s="4" t="s">
+      <c r="S6" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="S6" s="4" t="s">
+      <c r="T6" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -1452,7 +1485,7 @@
         <v>0.5</v>
       </c>
       <c r="F5" s="2">
-        <v>30000</v>
+        <v>15000</v>
       </c>
       <c r="G5" s="2">
         <v>8</v>

</xml_diff>